<commit_message>
Add script to auto-fill test checklist from pytest results
- scripts/update_excel_from_pytest.py: runs pytest --json-report and
  writes Pass/Fail + actual status code into the matching "Mã TC" rows
  of docs/Checklist_Test_API.xlsx (Kết quả thực tế, Pass/Fail, Người
  test, Ngày test columns), matching the existing dropdown/conditional
  formatting values.
- requirements.txt: add pytest-json-report, pytest-metadata.
- .gitignore: ignore the temporary .pytest_report.json.
- docs/Checklist_Test_API.xlsx: ran the script once, 77 mapped Mã TC
  rows filled in (66/66 pytest tests passing).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Checklist_Test_API.xlsx
+++ b/docs/Checklist_Test_API.xlsx
@@ -32,7 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="10">
     <font>
       <name val="Calibri"/>
@@ -139,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -160,6 +162,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1110,6 +1115,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -1284,10 +1290,24 @@
           <t>Trả về JSON báo trạng thái OK (vd. {"status":"ok"}), route này KHÔNG bọc envelope chuẩn</t>
         </is>
       </c>
-      <c r="O6" s="7" t="inlineStr"/>
-      <c r="P6" s="7" t="inlineStr"/>
-      <c r="Q6" s="7" t="inlineStr"/>
-      <c r="R6" s="7" t="inlineStr"/>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_health, PASS)</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R6" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S6" s="7" t="inlineStr">
         <is>
           <t>Dùng để xác nhận môi trường sẵn sàng trước khi test các API khác</t>
@@ -1368,6 +1388,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -1542,10 +1563,24 @@
           <t>data trả về UserOut (id, email, full_name, role=MEMBER mặc định, is_active=true, created_at); KHÔNG trả password_hash</t>
         </is>
       </c>
-      <c r="O6" s="7" t="inlineStr"/>
-      <c r="P6" s="7" t="inlineStr"/>
-      <c r="Q6" s="7" t="inlineStr"/>
-      <c r="R6" s="7" t="inlineStr"/>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>201 — khớp kỳ vọng (pytest: test_register_success, PASS)</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R6" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
@@ -1617,10 +1652,24 @@
           <t>message/error = "Email đã tồn tại"</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr"/>
-      <c r="P7" s="7" t="inlineStr"/>
-      <c r="Q7" s="7" t="inlineStr"/>
-      <c r="R7" s="7" t="inlineStr"/>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>400 — khớp kỳ vọng (pytest: test_register_duplicate_email, PASS)</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R7" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1767,10 +1816,24 @@
           <t>error chứa chi tiết field 'password' (min_length=6)</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr"/>
-      <c r="P9" s="7" t="inlineStr"/>
-      <c r="Q9" s="7" t="inlineStr"/>
-      <c r="R9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>422 — khớp kỳ vọng (pytest: test_register_password_too_short, PASS)</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q9" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
@@ -2001,10 +2064,24 @@
           <t>Trả thẳng {access_token, refresh_token, token_type="bearer"} — KHÔNG bọc envelope</t>
         </is>
       </c>
-      <c r="O13" s="7" t="inlineStr"/>
-      <c r="P13" s="7" t="inlineStr"/>
-      <c r="Q13" s="7" t="inlineStr"/>
-      <c r="R13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_login_success_returns_access_and_refresh_token, PASS)</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q13" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S13" s="7" t="inlineStr">
         <is>
           <t>Field 'username' trong form phải truyền EMAIL, không phải username thường</t>
@@ -2080,10 +2157,24 @@
           <t>message = "Sai email hoặc mật khẩu", header WWW-Authenticate: Bearer</t>
         </is>
       </c>
-      <c r="O14" s="7" t="inlineStr"/>
-      <c r="P14" s="7" t="inlineStr"/>
-      <c r="Q14" s="7" t="inlineStr"/>
-      <c r="R14" s="7" t="inlineStr"/>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>401 — khớp kỳ vọng (pytest: test_login_wrong_password, PASS)</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q14" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
@@ -2230,10 +2321,24 @@
           <t>message = "Tài khoản đã bị vô hiệu hóa, vui lòng liên hệ quản trị viên"</t>
         </is>
       </c>
-      <c r="O16" s="7" t="inlineStr"/>
-      <c r="P16" s="7" t="inlineStr"/>
-      <c r="Q16" s="7" t="inlineStr"/>
-      <c r="R16" s="7" t="inlineStr"/>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_login_inactive_account, PASS)</t>
+        </is>
+      </c>
+      <c r="P16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q16" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
@@ -2381,10 +2486,24 @@
           <t>message = "Bạn đã thử đăng nhập quá nhiều lần, vui lòng thử lại sau ít phút."</t>
         </is>
       </c>
-      <c r="O18" s="7" t="inlineStr"/>
-      <c r="P18" s="7" t="inlineStr"/>
-      <c r="Q18" s="7" t="inlineStr"/>
-      <c r="R18" s="7" t="inlineStr"/>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>429 — khớp kỳ vọng (pytest: test_login_rate_limit_blocks_after_max_attempts, PASS)</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q18" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R18" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S18" s="7" t="inlineStr">
         <is>
           <t>Giới hạn tính theo IP client (in-memory, không chia sẻ giữa nhiều worker) — set qua LOGIN_RATE_LIMIT_MAX_ATTEMPTS/WINDOW_SECONDS</t>
@@ -2467,10 +2586,24 @@
           <t>Trả thẳng access_token + refresh_token MỚI, token_type="bearer" — KHÔNG bọc envelope</t>
         </is>
       </c>
-      <c r="O20" s="7" t="inlineStr"/>
-      <c r="P20" s="7" t="inlineStr"/>
-      <c r="Q20" s="7" t="inlineStr"/>
-      <c r="R20" s="7" t="inlineStr"/>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_refresh_token_issues_new_access_token, PASS)</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q20" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
@@ -2692,10 +2825,24 @@
           <t>message = "Refresh token không hợp lệ" (do payload.type != "refresh")</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr"/>
-      <c r="P23" s="7" t="inlineStr"/>
-      <c r="Q23" s="7" t="inlineStr"/>
-      <c r="R23" s="7" t="inlineStr"/>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>401 — khớp kỳ vọng (pytest: test_refresh_rejects_access_token, PASS)</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q23" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
@@ -2925,6 +3072,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -3099,10 +3247,24 @@
           <t>data = UserOut của chính user đang đăng nhập</t>
         </is>
       </c>
-      <c r="O6" s="7" t="inlineStr"/>
-      <c r="P6" s="7" t="inlineStr"/>
-      <c r="Q6" s="7" t="inlineStr"/>
-      <c r="R6" s="7" t="inlineStr"/>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_get_current_user, PASS)</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R6" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
@@ -3174,10 +3336,24 @@
           <t>message mặc định của FastAPI OAuth2PasswordBearer ("Not authenticated")</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr"/>
-      <c r="P7" s="7" t="inlineStr"/>
-      <c r="Q7" s="7" t="inlineStr"/>
-      <c r="R7" s="7" t="inlineStr"/>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>401 — khớp kỳ vọng (pytest: test_get_current_user_without_token, PASS)</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R7" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -3249,10 +3425,24 @@
           <t>message = "Token đã hết hạn, vui lòng đăng nhập lại"</t>
         </is>
       </c>
-      <c r="O8" s="7" t="inlineStr"/>
-      <c r="P8" s="7" t="inlineStr"/>
-      <c r="Q8" s="7" t="inlineStr"/>
-      <c r="R8" s="7" t="inlineStr"/>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>401 — khớp kỳ vọng (pytest: test_get_current_user_expired_token, PASS)</t>
+        </is>
+      </c>
+      <c r="P8" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q8" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R8" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
@@ -3324,10 +3514,24 @@
           <t>message = "Token không hợp lệ"</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr"/>
-      <c r="P9" s="7" t="inlineStr"/>
-      <c r="Q9" s="7" t="inlineStr"/>
-      <c r="R9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>401 — khớp kỳ vọng (pytest: test_get_current_user_invalid_token, PASS)</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q9" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -3407,10 +3611,24 @@
           <t>data = danh sách toàn bộ UserOut</t>
         </is>
       </c>
-      <c r="O11" s="7" t="inlineStr"/>
-      <c r="P11" s="7" t="inlineStr"/>
-      <c r="Q11" s="7" t="inlineStr"/>
-      <c r="R11" s="7" t="inlineStr"/>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_users_as_admin_with_search_and_status_filter, PASS)</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q11" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
@@ -3482,10 +3700,24 @@
           <t>data chỉ gồm user có full_name hoặc email chứa 'nguyen' (không phân biệt hoa/thường)</t>
         </is>
       </c>
-      <c r="O12" s="7" t="inlineStr"/>
-      <c r="P12" s="7" t="inlineStr"/>
-      <c r="Q12" s="7" t="inlineStr"/>
-      <c r="R12" s="7" t="inlineStr"/>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_users_as_admin_with_search_and_status_filter, PASS)</t>
+        </is>
+      </c>
+      <c r="P12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q12" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
@@ -3557,10 +3789,24 @@
           <t>data chỉ gồm user có is_active=false</t>
         </is>
       </c>
-      <c r="O13" s="7" t="inlineStr"/>
-      <c r="P13" s="7" t="inlineStr"/>
-      <c r="Q13" s="7" t="inlineStr"/>
-      <c r="R13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_users_as_admin_with_search_and_status_filter, PASS)</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q13" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
@@ -3633,10 +3879,24 @@
           <t>message = "Bạn không có quyền thực hiện hành động này"</t>
         </is>
       </c>
-      <c r="O14" s="7" t="inlineStr"/>
-      <c r="P14" s="7" t="inlineStr"/>
-      <c r="Q14" s="7" t="inlineStr"/>
-      <c r="R14" s="7" t="inlineStr"/>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_list_users_requires_admin, PASS)</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q14" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
@@ -3789,6 +4049,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -3963,10 +4224,24 @@
           <t>data = SiteOut (id, name, description, owner_id = id của User B, created_at); User B tự động thành OWNER</t>
         </is>
       </c>
-      <c r="O6" s="7" t="inlineStr"/>
-      <c r="P6" s="7" t="inlineStr"/>
-      <c r="Q6" s="7" t="inlineStr"/>
-      <c r="R6" s="7" t="inlineStr"/>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>201 — khớp kỳ vọng (pytest: test_create_site_success_and_becomes_owner, PASS)</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R6" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
@@ -4113,10 +4388,24 @@
           <t>error field 'name' (min_length=1)</t>
         </is>
       </c>
-      <c r="O8" s="7" t="inlineStr"/>
-      <c r="P8" s="7" t="inlineStr"/>
-      <c r="Q8" s="7" t="inlineStr"/>
-      <c r="R8" s="7" t="inlineStr"/>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>422 — khớp kỳ vọng (pytest: test_create_site_name_blank_rejected, PASS)</t>
+        </is>
+      </c>
+      <c r="P8" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q8" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R8" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
@@ -4188,10 +4477,24 @@
           <t>Not authenticated</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr"/>
-      <c r="P9" s="7" t="inlineStr"/>
-      <c r="Q9" s="7" t="inlineStr"/>
-      <c r="R9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>401 — khớp kỳ vọng (pytest: test_create_site_requires_auth, PASS)</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q9" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
@@ -4263,10 +4566,24 @@
           <t>data chỉ gồm công trình mà User B là owner/member, không thấy công trình của user khác</t>
         </is>
       </c>
-      <c r="O10" s="7" t="inlineStr"/>
-      <c r="P10" s="7" t="inlineStr"/>
-      <c r="Q10" s="7" t="inlineStr"/>
-      <c r="R10" s="7" t="inlineStr"/>
+      <c r="O10" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_sites_only_returns_owner_or_member, PASS)</t>
+        </is>
+      </c>
+      <c r="P10" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q10" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R10" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
@@ -4338,10 +4655,24 @@
           <t>data chỉ gồm công trình có tên chứa từ khóa</t>
         </is>
       </c>
-      <c r="O11" s="7" t="inlineStr"/>
-      <c r="P11" s="7" t="inlineStr"/>
-      <c r="Q11" s="7" t="inlineStr"/>
-      <c r="R11" s="7" t="inlineStr"/>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_sites_search_by_name, PASS)</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q11" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
@@ -4563,10 +4894,24 @@
           <t>message = "Không tìm thấy công trình"</t>
         </is>
       </c>
-      <c r="O14" s="7" t="inlineStr"/>
-      <c r="P14" s="7" t="inlineStr"/>
-      <c r="Q14" s="7" t="inlineStr"/>
-      <c r="R14" s="7" t="inlineStr"/>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>404 — khớp kỳ vọng (pytest: test_get_site_not_found, PASS)</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q14" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
@@ -4638,10 +4983,24 @@
           <t>message = "Bạn không phải thành viên của công trình này"</t>
         </is>
       </c>
-      <c r="O15" s="7" t="inlineStr"/>
-      <c r="P15" s="7" t="inlineStr"/>
-      <c r="Q15" s="7" t="inlineStr"/>
-      <c r="R15" s="7" t="inlineStr"/>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_get_site_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q15" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
@@ -4713,10 +5072,24 @@
           <t>message = "Không tìm thấy công trình" (soft-delete bị filter khỏi query)</t>
         </is>
       </c>
-      <c r="O16" s="7" t="inlineStr"/>
-      <c r="P16" s="7" t="inlineStr"/>
-      <c r="Q16" s="7" t="inlineStr"/>
-      <c r="R16" s="7" t="inlineStr"/>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t>404 — khớp kỳ vọng (pytest: test_delete_site_soft_delete_hides_it, PASS)</t>
+        </is>
+      </c>
+      <c r="P16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q16" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
@@ -4788,10 +5161,24 @@
           <t>data.name đã được cập nhật; các field không gửi giữ nguyên</t>
         </is>
       </c>
-      <c r="O17" s="7" t="inlineStr"/>
-      <c r="P17" s="7" t="inlineStr"/>
-      <c r="Q17" s="7" t="inlineStr"/>
-      <c r="R17" s="7" t="inlineStr"/>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_update_site_owner_only, PASS)</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q17" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R17" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
@@ -4863,10 +5250,24 @@
           <t>data.name đã được cập nhật</t>
         </is>
       </c>
-      <c r="O18" s="7" t="inlineStr"/>
-      <c r="P18" s="7" t="inlineStr"/>
-      <c r="Q18" s="7" t="inlineStr"/>
-      <c r="R18" s="7" t="inlineStr"/>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_update_site_via_put_same_as_patch, PASS)</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q18" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R18" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
@@ -4938,10 +5339,24 @@
           <t>message = "Chỉ chủ sở hữu công trình mới được thực hiện hành động này"</t>
         </is>
       </c>
-      <c r="O19" s="7" t="inlineStr"/>
-      <c r="P19" s="7" t="inlineStr"/>
-      <c r="Q19" s="7" t="inlineStr"/>
-      <c r="R19" s="7" t="inlineStr"/>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_update_site_owner_only, PASS)</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q19" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R19" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
@@ -5164,10 +5579,24 @@
           <t>message thành công; GET lại site sau đó trả 404 (đã soft-delete, is_deleted=true)</t>
         </is>
       </c>
-      <c r="O22" s="7" t="inlineStr"/>
-      <c r="P22" s="7" t="inlineStr"/>
-      <c r="Q22" s="7" t="inlineStr"/>
-      <c r="R22" s="7" t="inlineStr"/>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_delete_site_soft_delete_hides_it, PASS)</t>
+        </is>
+      </c>
+      <c r="P22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q22" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R22" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
@@ -5239,10 +5668,24 @@
           <t>message = "Chỉ chủ sở hữu công trình mới được thực hiện hành động này"</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr"/>
-      <c r="P23" s="7" t="inlineStr"/>
-      <c r="Q23" s="7" t="inlineStr"/>
-      <c r="R23" s="7" t="inlineStr"/>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_delete_site_non_owner_forbidden, PASS)</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q23" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
@@ -5546,10 +5989,24 @@
           <t>data = SiteMemberOut với user_id, role=MEMBER, joined_at</t>
         </is>
       </c>
-      <c r="O28" s="7" t="inlineStr"/>
-      <c r="P28" s="7" t="inlineStr"/>
-      <c r="Q28" s="7" t="inlineStr"/>
-      <c r="R28" s="7" t="inlineStr"/>
+      <c r="O28" s="7" t="inlineStr">
+        <is>
+          <t>201 — khớp kỳ vọng (pytest: test_add_member_success_and_duplicate_rejected, PASS)</t>
+        </is>
+      </c>
+      <c r="P28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q28" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R28" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
@@ -5696,10 +6153,24 @@
           <t>message = "Người dùng đã là thành viên của công trình này"</t>
         </is>
       </c>
-      <c r="O30" s="7" t="inlineStr"/>
-      <c r="P30" s="7" t="inlineStr"/>
-      <c r="Q30" s="7" t="inlineStr"/>
-      <c r="R30" s="7" t="inlineStr"/>
+      <c r="O30" s="7" t="inlineStr">
+        <is>
+          <t>400 — khớp kỳ vọng (pytest: test_add_member_success_and_duplicate_rejected, PASS)</t>
+        </is>
+      </c>
+      <c r="P30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q30" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R30" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S30" s="7" t="inlineStr"/>
     </row>
     <row r="31">
@@ -5771,10 +6242,24 @@
           <t>message = "Không tìm thấy người dùng"</t>
         </is>
       </c>
-      <c r="O31" s="7" t="inlineStr"/>
-      <c r="P31" s="7" t="inlineStr"/>
-      <c r="Q31" s="7" t="inlineStr"/>
-      <c r="R31" s="7" t="inlineStr"/>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t>404 — khớp kỳ vọng (pytest: test_add_member_user_not_found, PASS)</t>
+        </is>
+      </c>
+      <c r="P31" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q31" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R31" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
@@ -5846,10 +6331,24 @@
           <t>message = "Chỉ chủ sở hữu công trình mới được thực hiện hành động này"</t>
         </is>
       </c>
-      <c r="O32" s="7" t="inlineStr"/>
-      <c r="P32" s="7" t="inlineStr"/>
-      <c r="Q32" s="7" t="inlineStr"/>
-      <c r="R32" s="7" t="inlineStr"/>
+      <c r="O32" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_add_member_non_owner_forbidden, PASS)</t>
+        </is>
+      </c>
+      <c r="P32" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q32" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R32" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S32" s="7" t="inlineStr"/>
     </row>
     <row r="33">
@@ -5996,10 +6495,24 @@
           <t>message thành công; GET lại danh sách members không còn User C</t>
         </is>
       </c>
-      <c r="O34" s="7" t="inlineStr"/>
-      <c r="P34" s="7" t="inlineStr"/>
-      <c r="Q34" s="7" t="inlineStr"/>
-      <c r="R34" s="7" t="inlineStr"/>
+      <c r="O34" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_remove_member_success, PASS)</t>
+        </is>
+      </c>
+      <c r="P34" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q34" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R34" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S34" s="7" t="inlineStr"/>
     </row>
     <row r="35">
@@ -6071,10 +6584,24 @@
           <t>message = "Không thể xóa chủ sở hữu cuối cùng của công trình"</t>
         </is>
       </c>
-      <c r="O35" s="7" t="inlineStr"/>
-      <c r="P35" s="7" t="inlineStr"/>
-      <c r="Q35" s="7" t="inlineStr"/>
-      <c r="R35" s="7" t="inlineStr"/>
+      <c r="O35" s="7" t="inlineStr">
+        <is>
+          <t>400 — khớp kỳ vọng (pytest: test_cannot_remove_last_owner, PASS)</t>
+        </is>
+      </c>
+      <c r="P35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q35" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R35" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
@@ -6146,10 +6673,24 @@
           <t>message = "Không tìm thấy thành viên trong công trình này"</t>
         </is>
       </c>
-      <c r="O36" s="7" t="inlineStr"/>
-      <c r="P36" s="7" t="inlineStr"/>
-      <c r="Q36" s="7" t="inlineStr"/>
-      <c r="R36" s="7" t="inlineStr"/>
+      <c r="O36" s="7" t="inlineStr">
+        <is>
+          <t>404 — khớp kỳ vọng (pytest: test_remove_member_not_found, PASS)</t>
+        </is>
+      </c>
+      <c r="P36" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q36" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R36" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
@@ -6302,6 +6843,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -6475,10 +7017,24 @@
           <t>data = TeamOut (id, site_id, name, description, created_at)</t>
         </is>
       </c>
-      <c r="O6" s="7" t="inlineStr"/>
-      <c r="P6" s="7" t="inlineStr"/>
-      <c r="Q6" s="7" t="inlineStr"/>
-      <c r="R6" s="7" t="inlineStr"/>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>201 — khớp kỳ vọng (pytest: test_create_team_owner_only, PASS)</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R6" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
@@ -6550,10 +7106,24 @@
           <t>message = "Chỉ chủ sở hữu công trình mới được thực hiện hành động này"</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr"/>
-      <c r="P7" s="7" t="inlineStr"/>
-      <c r="Q7" s="7" t="inlineStr"/>
-      <c r="R7" s="7" t="inlineStr"/>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_create_team_owner_only, PASS)</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R7" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -6850,10 +7420,24 @@
           <t>message = "Bạn không phải thành viên của công trình này"</t>
         </is>
       </c>
-      <c r="O11" s="7" t="inlineStr"/>
-      <c r="P11" s="7" t="inlineStr"/>
-      <c r="Q11" s="7" t="inlineStr"/>
-      <c r="R11" s="7" t="inlineStr"/>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_team_list_requires_site_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q11" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R11" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
@@ -6925,10 +7509,24 @@
           <t>data = TeamOut đầy đủ</t>
         </is>
       </c>
-      <c r="O12" s="7" t="inlineStr"/>
-      <c r="P12" s="7" t="inlineStr"/>
-      <c r="Q12" s="7" t="inlineStr"/>
-      <c r="R12" s="7" t="inlineStr"/>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_get_team_detail_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q12" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
@@ -7000,10 +7598,24 @@
           <t>message = "Không tìm thấy đội thi công"</t>
         </is>
       </c>
-      <c r="O13" s="7" t="inlineStr"/>
-      <c r="P13" s="7" t="inlineStr"/>
-      <c r="Q13" s="7" t="inlineStr"/>
-      <c r="R13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>404 — khớp kỳ vọng (pytest: test_get_team_not_found, PASS)</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q13" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
@@ -7075,10 +7687,24 @@
           <t>data.name đã cập nhật</t>
         </is>
       </c>
-      <c r="O14" s="7" t="inlineStr"/>
-      <c r="P14" s="7" t="inlineStr"/>
-      <c r="Q14" s="7" t="inlineStr"/>
-      <c r="R14" s="7" t="inlineStr"/>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_update_team_owner_only, PASS)</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q14" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
@@ -7150,10 +7776,24 @@
           <t>message = "Chỉ chủ sở hữu công trình mới được thực hiện hành động này"</t>
         </is>
       </c>
-      <c r="O15" s="7" t="inlineStr"/>
-      <c r="P15" s="7" t="inlineStr"/>
-      <c r="Q15" s="7" t="inlineStr"/>
-      <c r="R15" s="7" t="inlineStr"/>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_update_team_owner_only, PASS)</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q15" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
@@ -7226,10 +7866,24 @@
           <t>message thành công; work item liên quan có assignee_team_id=null</t>
         </is>
       </c>
-      <c r="O16" s="7" t="inlineStr"/>
-      <c r="P16" s="7" t="inlineStr"/>
-      <c r="Q16" s="7" t="inlineStr"/>
-      <c r="R16" s="7" t="inlineStr"/>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_delete_team_owner_only_and_unassigns_work_items, PASS)</t>
+        </is>
+      </c>
+      <c r="P16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q16" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
@@ -7301,10 +7955,24 @@
           <t>message = "Chỉ chủ sở hữu công trình mới được thực hiện hành động này"</t>
         </is>
       </c>
-      <c r="O17" s="7" t="inlineStr"/>
-      <c r="P17" s="7" t="inlineStr"/>
-      <c r="Q17" s="7" t="inlineStr"/>
-      <c r="R17" s="7" t="inlineStr"/>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_delete_team_owner_only_and_unassigns_work_items, PASS)</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q17" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R17" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
@@ -7458,10 +8126,24 @@
           <t>data = danh sách TeamMemberOut</t>
         </is>
       </c>
-      <c r="O20" s="7" t="inlineStr"/>
-      <c r="P20" s="7" t="inlineStr"/>
-      <c r="Q20" s="7" t="inlineStr"/>
-      <c r="R20" s="7" t="inlineStr"/>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_team_members, PASS)</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q20" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
@@ -7608,10 +8290,24 @@
           <t>message = "Chỉ có thể thêm người đã là thành viên của công trình vào đội thi công"</t>
         </is>
       </c>
-      <c r="O22" s="7" t="inlineStr"/>
-      <c r="P22" s="7" t="inlineStr"/>
-      <c r="Q22" s="7" t="inlineStr"/>
-      <c r="R22" s="7" t="inlineStr"/>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>400 — khớp kỳ vọng (pytest: test_add_team_member_requires_site_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q22" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R22" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
@@ -7683,10 +8379,24 @@
           <t>message = "Người dùng đã thuộc đội thi công này"</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr"/>
-      <c r="P23" s="7" t="inlineStr"/>
-      <c r="Q23" s="7" t="inlineStr"/>
-      <c r="R23" s="7" t="inlineStr"/>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>400 — khớp kỳ vọng (pytest: test_add_team_member_duplicate_rejected, PASS)</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q23" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
@@ -7833,10 +8543,24 @@
           <t>message thành công; GET lại danh sách team members không còn User C</t>
         </is>
       </c>
-      <c r="O25" s="7" t="inlineStr"/>
-      <c r="P25" s="7" t="inlineStr"/>
-      <c r="Q25" s="7" t="inlineStr"/>
-      <c r="R25" s="7" t="inlineStr"/>
+      <c r="O25" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_remove_team_member_owner_only_and_not_found, PASS)</t>
+        </is>
+      </c>
+      <c r="P25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q25" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R25" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
@@ -7908,10 +8632,24 @@
           <t>message = "Không tìm thấy thành viên trong đội thi công này"</t>
         </is>
       </c>
-      <c r="O26" s="7" t="inlineStr"/>
-      <c r="P26" s="7" t="inlineStr"/>
-      <c r="Q26" s="7" t="inlineStr"/>
-      <c r="R26" s="7" t="inlineStr"/>
+      <c r="O26" s="7" t="inlineStr">
+        <is>
+          <t>404 — khớp kỳ vọng (pytest: test_remove_team_member_owner_only_and_not_found, PASS)</t>
+        </is>
+      </c>
+      <c r="P26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q26" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R26" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S26" s="7" t="inlineStr"/>
     </row>
   </sheetData>
@@ -7990,6 +8728,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -8163,10 +8902,24 @@
           <t>data = WorkItemOut, status mặc định=TODO, assignee_team lồng thông tin Team Y</t>
         </is>
       </c>
-      <c r="O6" s="7" t="inlineStr"/>
-      <c r="P6" s="7" t="inlineStr"/>
-      <c r="Q6" s="7" t="inlineStr"/>
-      <c r="R6" s="7" t="inlineStr"/>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>201 — khớp kỳ vọng (pytest: test_create_work_item_with_valid_assignee_team, PASS)</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R6" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
@@ -8313,10 +9066,24 @@
           <t>message = "Đội thi công không tồn tại hoặc không thuộc công trình này"</t>
         </is>
       </c>
-      <c r="O8" s="7" t="inlineStr"/>
-      <c r="P8" s="7" t="inlineStr"/>
-      <c r="Q8" s="7" t="inlineStr"/>
-      <c r="R8" s="7" t="inlineStr"/>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>400 — khớp kỳ vọng (pytest: test_create_work_item_assignee_team_must_belong_to_site, PASS)</t>
+        </is>
+      </c>
+      <c r="P8" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q8" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R8" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
@@ -8388,10 +9155,24 @@
           <t>message = "Bạn không phải thành viên của công trình này"</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr"/>
-      <c r="P9" s="7" t="inlineStr"/>
-      <c r="Q9" s="7" t="inlineStr"/>
-      <c r="R9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_create_work_item_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q9" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R9" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
@@ -8613,10 +9394,24 @@
           <t>data = {items:[...], total, page=1, size=20}</t>
         </is>
       </c>
-      <c r="O12" s="7" t="inlineStr"/>
-      <c r="P12" s="7" t="inlineStr"/>
-      <c r="Q12" s="7" t="inlineStr"/>
-      <c r="R12" s="7" t="inlineStr"/>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_work_items_scoped_to_site, PASS)</t>
+        </is>
+      </c>
+      <c r="P12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q12" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
@@ -8688,10 +9483,24 @@
           <t>items chỉ gồm hạng mục có status=TODO và priority=HIGH</t>
         </is>
       </c>
-      <c r="O13" s="7" t="inlineStr"/>
-      <c r="P13" s="7" t="inlineStr"/>
-      <c r="Q13" s="7" t="inlineStr"/>
-      <c r="R13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_work_items_filter_and_search, PASS)</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q13" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
@@ -8763,10 +9572,24 @@
           <t>items chứa từ khóa trong title, sắp xếp due_date tăng dần</t>
         </is>
       </c>
-      <c r="O14" s="7" t="inlineStr"/>
-      <c r="P14" s="7" t="inlineStr"/>
-      <c r="Q14" s="7" t="inlineStr"/>
-      <c r="R14" s="7" t="inlineStr"/>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_work_items_filter_and_search, PASS)</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q14" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R14" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
@@ -8838,10 +9661,24 @@
           <t>items trả về đúng 1 phần tử (bản ghi thứ 2), total đúng tổng số</t>
         </is>
       </c>
-      <c r="O15" s="7" t="inlineStr"/>
-      <c r="P15" s="7" t="inlineStr"/>
-      <c r="Q15" s="7" t="inlineStr"/>
-      <c r="R15" s="7" t="inlineStr"/>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_work_items_pagination, PASS)</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q15" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
@@ -9064,10 +9901,24 @@
           <t>items chỉ gồm hạng mục thuộc đúng site_id truyền vào</t>
         </is>
       </c>
-      <c r="O18" s="7" t="inlineStr"/>
-      <c r="P18" s="7" t="inlineStr"/>
-      <c r="Q18" s="7" t="inlineStr"/>
-      <c r="R18" s="7" t="inlineStr"/>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_list_work_items_scoped_to_site, PASS)</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q18" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R18" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
@@ -9139,10 +9990,24 @@
           <t>data = WorkItemOut đầy đủ, có lồng assignee_team</t>
         </is>
       </c>
-      <c r="O19" s="7" t="inlineStr"/>
-      <c r="P19" s="7" t="inlineStr"/>
-      <c r="Q19" s="7" t="inlineStr"/>
-      <c r="R19" s="7" t="inlineStr"/>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_get_work_item_detail_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q19" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R19" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
@@ -9214,10 +10079,24 @@
           <t>message = "Không tìm thấy hạng mục thi công"</t>
         </is>
       </c>
-      <c r="O20" s="7" t="inlineStr"/>
-      <c r="P20" s="7" t="inlineStr"/>
-      <c r="Q20" s="7" t="inlineStr"/>
-      <c r="R20" s="7" t="inlineStr"/>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>404 — khớp kỳ vọng (pytest: test_get_work_item_not_found, PASS)</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q20" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
@@ -9289,10 +10168,24 @@
           <t>message = "Bạn không phải thành viên của công trình này"</t>
         </is>
       </c>
-      <c r="O21" s="7" t="inlineStr"/>
-      <c r="P21" s="7" t="inlineStr"/>
-      <c r="Q21" s="7" t="inlineStr"/>
-      <c r="R21" s="7" t="inlineStr"/>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_get_work_item_detail_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q21" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
@@ -9364,10 +10257,24 @@
           <t>data phản ánh đúng field đã sửa</t>
         </is>
       </c>
-      <c r="O22" s="7" t="inlineStr"/>
-      <c r="P22" s="7" t="inlineStr"/>
-      <c r="Q22" s="7" t="inlineStr"/>
-      <c r="R22" s="7" t="inlineStr"/>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_update_work_item_owner_can_edit_any_field, PASS)</t>
+        </is>
+      </c>
+      <c r="P22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q22" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R22" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
@@ -9439,10 +10346,24 @@
           <t>data.status/description cập nhật thành công</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr"/>
-      <c r="P23" s="7" t="inlineStr"/>
-      <c r="Q23" s="7" t="inlineStr"/>
-      <c r="R23" s="7" t="inlineStr"/>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_update_work_item_assignee_team_member_can_only_update_status_description, PASS)</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q23" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
@@ -9514,10 +10435,24 @@
           <t>message = "Chỉ chủ sở hữu công trình mới được sửa title/priority/due_date/assignee_team_id"</t>
         </is>
       </c>
-      <c r="O24" s="7" t="inlineStr"/>
-      <c r="P24" s="7" t="inlineStr"/>
-      <c r="Q24" s="7" t="inlineStr"/>
-      <c r="R24" s="7" t="inlineStr"/>
+      <c r="O24" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_update_work_item_assignee_team_member_can_only_update_status_description, PASS)</t>
+        </is>
+      </c>
+      <c r="P24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q24" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R24" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
@@ -9589,10 +10524,24 @@
           <t>message = "Bạn không có quyền cập nhật hạng mục thi công này"</t>
         </is>
       </c>
-      <c r="O25" s="7" t="inlineStr"/>
-      <c r="P25" s="7" t="inlineStr"/>
-      <c r="Q25" s="7" t="inlineStr"/>
-      <c r="R25" s="7" t="inlineStr"/>
+      <c r="O25" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_update_work_item_unrelated_member_forbidden, PASS)</t>
+        </is>
+      </c>
+      <c r="P25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q25" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R25" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
@@ -9815,10 +10764,24 @@
           <t>message thành công; GET lại trả 404</t>
         </is>
       </c>
-      <c r="O28" s="7" t="inlineStr"/>
-      <c r="P28" s="7" t="inlineStr"/>
-      <c r="Q28" s="7" t="inlineStr"/>
-      <c r="R28" s="7" t="inlineStr"/>
+      <c r="O28" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_delete_work_item_owner_only, PASS)</t>
+        </is>
+      </c>
+      <c r="P28" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q28" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R28" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
@@ -9890,10 +10853,24 @@
           <t>message = "Chỉ chủ sở hữu công trình mới được xóa hạng mục thi công"</t>
         </is>
       </c>
-      <c r="O29" s="7" t="inlineStr"/>
-      <c r="P29" s="7" t="inlineStr"/>
-      <c r="Q29" s="7" t="inlineStr"/>
-      <c r="R29" s="7" t="inlineStr"/>
+      <c r="O29" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_delete_work_item_owner_only, PASS)</t>
+        </is>
+      </c>
+      <c r="P29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q29" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R29" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
@@ -10045,6 +11022,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -10218,10 +11196,24 @@
           <t>data = danh sách comment sắp xếp theo created_at tăng dần, có thông tin user</t>
         </is>
       </c>
-      <c r="O6" s="7" t="inlineStr"/>
-      <c r="P6" s="7" t="inlineStr"/>
-      <c r="Q6" s="7" t="inlineStr"/>
-      <c r="R6" s="7" t="inlineStr"/>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_comment_create_and_list_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R6" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
@@ -10293,10 +11285,24 @@
           <t>message = "Bạn không phải thành viên của công trình này"</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr"/>
-      <c r="P7" s="7" t="inlineStr"/>
-      <c r="Q7" s="7" t="inlineStr"/>
-      <c r="R7" s="7" t="inlineStr"/>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_comment_create_and_list_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R7" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -10368,10 +11374,24 @@
           <t>data = WorkItemCommentOut gồm id, content, user (người viết), created_at</t>
         </is>
       </c>
-      <c r="O8" s="7" t="inlineStr"/>
-      <c r="P8" s="7" t="inlineStr"/>
-      <c r="Q8" s="7" t="inlineStr"/>
-      <c r="R8" s="7" t="inlineStr"/>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>201 — khớp kỳ vọng (pytest: test_comment_create_and_list_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P8" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q8" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R8" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
@@ -10668,10 +11688,24 @@
           <t>message = "Bạn không phải thành viên của công trình này"</t>
         </is>
       </c>
-      <c r="O12" s="7" t="inlineStr"/>
-      <c r="P12" s="7" t="inlineStr"/>
-      <c r="Q12" s="7" t="inlineStr"/>
-      <c r="R12" s="7" t="inlineStr"/>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_comment_create_and_list_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q12" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R12" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -10825,10 +11859,24 @@
           <t>data.content_type = "application/pdf"</t>
         </is>
       </c>
-      <c r="O15" s="7" t="inlineStr"/>
-      <c r="P15" s="7" t="inlineStr"/>
-      <c r="Q15" s="7" t="inlineStr"/>
-      <c r="R15" s="7" t="inlineStr"/>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>201 — khớp kỳ vọng (pytest: test_upload_attachment_success_and_list, PASS)</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q15" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R15" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
@@ -10900,10 +11948,24 @@
           <t>message = "Loại file không được hỗ trợ, chỉ chấp nhận ảnh (jpg/png/webp) hoặc PDF"</t>
         </is>
       </c>
-      <c r="O16" s="7" t="inlineStr"/>
-      <c r="P16" s="7" t="inlineStr"/>
-      <c r="Q16" s="7" t="inlineStr"/>
-      <c r="R16" s="7" t="inlineStr"/>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t>400 — khớp kỳ vọng (pytest: test_upload_attachment_rejects_invalid_type, PASS)</t>
+        </is>
+      </c>
+      <c r="P16" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q16" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
@@ -11200,10 +12262,24 @@
           <t>message = "Bạn không phải thành viên của công trình này"</t>
         </is>
       </c>
-      <c r="O20" s="7" t="inlineStr"/>
-      <c r="P20" s="7" t="inlineStr"/>
-      <c r="Q20" s="7" t="inlineStr"/>
-      <c r="R20" s="7" t="inlineStr"/>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>403 — khớp kỳ vọng (pytest: test_upload_attachment_requires_membership, PASS)</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q20" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R20" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
@@ -11275,10 +12351,24 @@
           <t>data = danh sách attachment sắp xếp theo created_at tăng dần</t>
         </is>
       </c>
-      <c r="O21" s="7" t="inlineStr"/>
-      <c r="P21" s="7" t="inlineStr"/>
-      <c r="Q21" s="7" t="inlineStr"/>
-      <c r="R21" s="7" t="inlineStr"/>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>200 — khớp kỳ vọng (pytest: test_upload_attachment_success_and_list, PASS)</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q21" s="7" t="inlineStr">
+        <is>
+          <t>pytest (tự động)</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="n">
+        <v>46260</v>
+      </c>
       <c r="S21" s="7" t="inlineStr"/>
     </row>
     <row r="22">

</xml_diff>